<commit_message>
Update pipeline: ffill before zscore, rolling zscore for fusion normalization
- Move ffill from after pairwise diff to before rolling z-score (02, 03, 04)
- Replace full-sample std normalization with rolling z-score before fusion (04)
- Config: ROLLING_ZSCORE_WINDOW=90, MIN_VALID=90, PVALUE=0.05

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/factor_build/outputs/04_fusion_constituents.xlsx
+++ b/factor_build/outputs/04_fusion_constituents.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,13 +467,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-0.06610000000000001</v>
+        <v>-0.0616</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="3">
@@ -484,17 +484,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>510050.SH-510100.SH</t>
+          <t>159915.SZ-159952.SZ</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.0806</v>
+        <v>-0.0969</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="4">
@@ -505,35 +505,35 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>588080.SH-588050.SH</t>
+          <t>159915.SZ-159977.SZ</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.0649</v>
+        <v>-0.0602</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>netinflow</t>
+          <t>NAV_iopv_discount</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>159915.SZ-159977.SZ</t>
+          <t>510050.SH-510100.SH</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-0.06610000000000001</v>
+        <v>0.2049</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -542,7 +542,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>netinflow</t>
+          <t>amt</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -551,10 +551,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.0664</v>
+        <v>0.1107</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
@@ -563,19 +563,19 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>pct_chg</t>
+          <t>amt_btin</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>159915.SZ-159977.SZ</t>
+          <t>588080.SH-588050.SH</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-0.0578</v>
+        <v>0.1111</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>1</v>
@@ -584,21 +584,189 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>pct_chg</t>
+          <t>iopv</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>159915.SZ-159952.SZ</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0528</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>netinflow</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>159915.SZ-159977.SZ</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.0737</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>netinflow</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>588080.SH-588050.SH</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.0689</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>turn</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>510050.SH-510100.SH</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>0.0588</v>
-      </c>
-      <c r="D8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E8" t="n">
+      <c r="C11" t="n">
+        <v>0.0537</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>turn</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>588080.SH-588050.SH</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.1233</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>volume</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>510050.SH-510100.SH</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.0573</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>volume</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>588080.SH-588050.SH</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.1138</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>volume_btin</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>510050.SH-510100.SH</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.0562</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>volume_btin</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>588080.SH-588050.SH</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.1143</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Made all factors more rational
</commit_message>
<xml_diff>
--- a/factor_build/outputs/04_fusion_constituents.xlsx
+++ b/factor_build/outputs/04_fusion_constituents.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ETF申购赎回现金差额</t>
+          <t>NAV_iopv_discount</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -467,19 +467,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-0.0616</v>
+        <v>0.2049</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NAV_iopv_discount</t>
+          <t>netinflow</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -488,285 +488,54 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.0969</v>
+        <v>0.0582</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="E3" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NAV_iopv_discount</t>
+          <t>turn</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>159915.SZ-159977.SZ</t>
+          <t>588080.SH-588050.SH</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-0.0602</v>
+        <v>0.1233</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NAV_iopv_discount</t>
+          <t>volume_btin</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>510050.SH-510100.SH</t>
+          <t>588080.SH-588050.SH</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.2049</v>
+        <v>0.1143</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>amt</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>588080.SH-588050.SH</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0.1107</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>amt_btin</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>588080.SH-588050.SH</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0.1111</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>iopv</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>159915.SZ-159952.SZ</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0.0528</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>netinflow</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>159915.SZ-159977.SZ</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>0.0737</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>netinflow</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>588080.SH-588050.SH</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>0.0689</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>turn</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>510050.SH-510100.SH</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>turn</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>588080.SH-588050.SH</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>0.1233</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>volume</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>510050.SH-510100.SH</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>0.0573</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>volume</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>588080.SH-588050.SH</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>0.1138</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>volume_btin</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>510050.SH-510100.SH</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>0.0562</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>volume_btin</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>588080.SH-588050.SH</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>0.1143</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>